<commit_message>
Show English words in Hindi and Punjabi until translations arrive
Phrases without a local translation now carry the English word in both
languages (marked as English placeholders in the sheet) so the app is
complete in all three languages and the sheet still flags what is left.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Kp58nu653YnJ2qCdF8F9v
</commit_message>
<xml_diff>
--- a/locale/translations.xlsx
+++ b/locale/translations.xlsx
@@ -850,11 +850,19 @@
           <t>Chain of custody</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Chain of custody</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Chain of custody</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1038,11 +1046,19 @@
           <t>Biomass Mitra</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitra</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitra</t>
+        </is>
+      </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1590,11 +1606,19 @@
           <t>Tamper-evident trail</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr"/>
-      <c r="C42" s="3" t="inlineStr"/>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Tamper-evident trail</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Tamper-evident trail</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -1610,11 +1634,19 @@
           <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr"/>
-      <c r="C43" s="3" t="inlineStr"/>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
+        </is>
+      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -1658,11 +1690,19 @@
           <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr"/>
-      <c r="C45" s="3" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
+        </is>
+      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2854,11 +2894,19 @@
           <t>Book inventory</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr"/>
-      <c r="C88" s="3" t="inlineStr"/>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Book inventory</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Book inventory</t>
+        </is>
+      </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2902,11 +2950,19 @@
           <t>Physical inventory</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr"/>
-      <c r="C90" s="3" t="inlineStr"/>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Physical inventory</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Physical inventory</t>
+        </is>
+      </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2950,11 +3006,19 @@
           <t>Usable inventory</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr"/>
-      <c r="C92" s="3" t="inlineStr"/>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Usable inventory</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Usable inventory</t>
+        </is>
+      </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2998,11 +3062,19 @@
           <t>Fuel cover</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr"/>
-      <c r="C94" s="3" t="inlineStr"/>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Fuel cover</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Fuel cover</t>
+        </is>
+      </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -3942,19 +4014,19 @@
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
-      <c r="B128" s="2" t="inlineStr">
+      <c r="B128" s="3" t="inlineStr">
         <is>
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
-      <c r="C128" s="2" t="inlineStr">
+      <c r="C128" s="3" t="inlineStr">
         <is>
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Draft: please check</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -4082,11 +4154,19 @@
           <t>Biomass Mitras</t>
         </is>
       </c>
-      <c r="B133" s="3" t="inlineStr"/>
-      <c r="C133" s="3" t="inlineStr"/>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitras</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitras</t>
+        </is>
+      </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
@@ -4102,11 +4182,19 @@
           <t>No Mitra recorded.</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr"/>
-      <c r="C134" s="3" t="inlineStr"/>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>No Mitra recorded.</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>No Mitra recorded.</t>
+        </is>
+      </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -4122,11 +4210,19 @@
           <t>Grids</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr"/>
-      <c r="C135" s="3" t="inlineStr"/>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Grids</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Grids</t>
+        </is>
+      </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
@@ -4142,11 +4238,19 @@
           <t>Attributed</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr"/>
-      <c r="C136" s="3" t="inlineStr"/>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Attributed</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Attributed</t>
+        </is>
+      </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -4190,11 +4294,19 @@
           <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr"/>
-      <c r="C138" s="3" t="inlineStr"/>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
+        </is>
+      </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -4238,11 +4350,19 @@
           <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr"/>
-      <c r="C140" s="3" t="inlineStr"/>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
+        </is>
+      </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -4342,11 +4462,19 @@
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr"/>
-      <c r="C144" s="3" t="inlineStr"/>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -4558,11 +4686,19 @@
           <t>ESG / sustainability</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr"/>
-      <c r="C152" s="3" t="inlineStr"/>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>ESG / sustainability</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>ESG / sustainability</t>
+        </is>
+      </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -4578,11 +4714,19 @@
           <t>Regenerix</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr"/>
-      <c r="C153" s="3" t="inlineStr"/>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Regenerix</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Regenerix</t>
+        </is>
+      </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -4598,11 +4742,19 @@
           <t>VLE</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr"/>
-      <c r="C154" s="3" t="inlineStr"/>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>VLE</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>VLE</t>
+        </is>
+      </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -5738,11 +5890,19 @@
           <t>Reconcile</t>
         </is>
       </c>
-      <c r="B195" s="3" t="inlineStr"/>
-      <c r="C195" s="3" t="inlineStr"/>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Reconcile</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Reconcile</t>
+        </is>
+      </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -5786,11 +5946,19 @@
           <t>Low fuel cover</t>
         </is>
       </c>
-      <c r="B197" s="3" t="inlineStr"/>
-      <c r="C197" s="3" t="inlineStr"/>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Low fuel cover</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>Low fuel cover</t>
+        </is>
+      </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -5806,11 +5974,19 @@
           <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
         </is>
       </c>
-      <c r="B198" s="3" t="inlineStr"/>
-      <c r="C198" s="3" t="inlineStr"/>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
+        </is>
+      </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -6106,11 +6282,19 @@
           <t>At the Grid</t>
         </is>
       </c>
-      <c r="B209" s="3" t="inlineStr"/>
-      <c r="C209" s="3" t="inlineStr"/>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>At the Grid</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>At the Grid</t>
+        </is>
+      </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
@@ -6126,11 +6310,19 @@
           <t>At the Hub</t>
         </is>
       </c>
-      <c r="B210" s="3" t="inlineStr"/>
-      <c r="C210" s="3" t="inlineStr"/>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>At the Hub</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>At the Hub</t>
+        </is>
+      </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -6171,7 +6363,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Blank: please supply,Draft: please check,Checked in the field,Needs discussion"</formula1>
+      <formula1>"English placeholder: please translate,Draft: please check,Checked in the field,Needs discussion"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6200,7 +6392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Column A is the English. Fill in or correct column B (Hindi) and column C (Punjabi). Yellow cells are blank because I was not sure of the local wording.</t>
+          <t>Column A is the English. Fill in or correct column B (Hindi) and column C (Punjabi). Yellow cells still show the English word because I was not sure of the local wording; please replace it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show English words in Hindi and Punjabi until translations arrive (#19)
Phrases without a local translation now carry the English word in both
languages (marked as English placeholders in the sheet) so the app is
complete in all three languages and the sheet still flags what is left.


Claude-Session: https://claude.ai/code/session_012Kp58nu653YnJ2qCdF8F9v

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/locale/translations.xlsx
+++ b/locale/translations.xlsx
@@ -850,11 +850,19 @@
           <t>Chain of custody</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Chain of custody</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Chain of custody</t>
+        </is>
+      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1038,11 +1046,19 @@
           <t>Biomass Mitra</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitra</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitra</t>
+        </is>
+      </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1590,11 +1606,19 @@
           <t>Tamper-evident trail</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr"/>
-      <c r="C42" s="3" t="inlineStr"/>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Tamper-evident trail</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Tamper-evident trail</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -1610,11 +1634,19 @@
           <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr"/>
-      <c r="C43" s="3" t="inlineStr"/>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Each entry carries a fingerprint of the one before it, so a changed record would be detected.</t>
+        </is>
+      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -1658,11 +1690,19 @@
           <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr"/>
-      <c r="C45" s="3" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Farmers: %(n)s. Shared out by what each handed over at the Grid. Codes and villages only.</t>
+        </is>
+      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2854,11 +2894,19 @@
           <t>Book inventory</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr"/>
-      <c r="C88" s="3" t="inlineStr"/>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Book inventory</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Book inventory</t>
+        </is>
+      </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2902,11 +2950,19 @@
           <t>Physical inventory</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr"/>
-      <c r="C90" s="3" t="inlineStr"/>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Physical inventory</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Physical inventory</t>
+        </is>
+      </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -2950,11 +3006,19 @@
           <t>Usable inventory</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr"/>
-      <c r="C92" s="3" t="inlineStr"/>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Usable inventory</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Usable inventory</t>
+        </is>
+      </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2998,11 +3062,19 @@
           <t>Fuel cover</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr"/>
-      <c r="C94" s="3" t="inlineStr"/>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Fuel cover</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Fuel cover</t>
+        </is>
+      </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -3942,19 +4014,19 @@
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
-      <c r="B128" s="2" t="inlineStr">
+      <c r="B128" s="3" t="inlineStr">
         <is>
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
-      <c r="C128" s="2" t="inlineStr">
+      <c r="C128" s="3" t="inlineStr">
         <is>
           <t>%(d)s (%(pc)s%%)</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Draft: please check</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -4082,11 +4154,19 @@
           <t>Biomass Mitras</t>
         </is>
       </c>
-      <c r="B133" s="3" t="inlineStr"/>
-      <c r="C133" s="3" t="inlineStr"/>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitras</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Biomass Mitras</t>
+        </is>
+      </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
@@ -4102,11 +4182,19 @@
           <t>No Mitra recorded.</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr"/>
-      <c r="C134" s="3" t="inlineStr"/>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>No Mitra recorded.</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>No Mitra recorded.</t>
+        </is>
+      </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -4122,11 +4210,19 @@
           <t>Grids</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr"/>
-      <c r="C135" s="3" t="inlineStr"/>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Grids</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Grids</t>
+        </is>
+      </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
@@ -4142,11 +4238,19 @@
           <t>Attributed</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr"/>
-      <c r="C136" s="3" t="inlineStr"/>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Attributed</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Attributed</t>
+        </is>
+      </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -4190,11 +4294,19 @@
           <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr"/>
-      <c r="C138" s="3" t="inlineStr"/>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s delivered. Farmers are shared out in proportion to the tonnes each handed over at the supplying Grid (the lots are not tagged farmer by farmer), so read this as a fair attribution, not lot-level proof. Only farmer codes and villages are shown.</t>
+        </is>
+      </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -4238,11 +4350,19 @@
           <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr"/>
-      <c r="C140" s="3" t="inlineStr"/>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>%(t)s could not be attributed because no farmer pickups are recorded for it.</t>
+        </is>
+      </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
@@ -4342,11 +4462,19 @@
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr"/>
-      <c r="C144" s="3" t="inlineStr"/>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -4558,11 +4686,19 @@
           <t>ESG / sustainability</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr"/>
-      <c r="C152" s="3" t="inlineStr"/>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>ESG / sustainability</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>ESG / sustainability</t>
+        </is>
+      </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -4578,11 +4714,19 @@
           <t>Regenerix</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr"/>
-      <c r="C153" s="3" t="inlineStr"/>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Regenerix</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Regenerix</t>
+        </is>
+      </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -4598,11 +4742,19 @@
           <t>VLE</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr"/>
-      <c r="C154" s="3" t="inlineStr"/>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>VLE</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>VLE</t>
+        </is>
+      </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -5738,11 +5890,19 @@
           <t>Reconcile</t>
         </is>
       </c>
-      <c r="B195" s="3" t="inlineStr"/>
-      <c r="C195" s="3" t="inlineStr"/>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Reconcile</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Reconcile</t>
+        </is>
+      </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -5786,11 +5946,19 @@
           <t>Low fuel cover</t>
         </is>
       </c>
-      <c r="B197" s="3" t="inlineStr"/>
-      <c r="C197" s="3" t="inlineStr"/>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Low fuel cover</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>Low fuel cover</t>
+        </is>
+      </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -5806,11 +5974,19 @@
           <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
         </is>
       </c>
-      <c r="B198" s="3" t="inlineStr"/>
-      <c r="C198" s="3" t="inlineStr"/>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>%(days)s days of cover is less than the %(lead)s-day replenishment lead time.</t>
+        </is>
+      </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -6106,11 +6282,19 @@
           <t>At the Grid</t>
         </is>
       </c>
-      <c r="B209" s="3" t="inlineStr"/>
-      <c r="C209" s="3" t="inlineStr"/>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>At the Grid</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>At the Grid</t>
+        </is>
+      </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
@@ -6126,11 +6310,19 @@
           <t>At the Hub</t>
         </is>
       </c>
-      <c r="B210" s="3" t="inlineStr"/>
-      <c r="C210" s="3" t="inlineStr"/>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>At the Hub</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>At the Hub</t>
+        </is>
+      </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>Blank: please supply</t>
+          <t>English placeholder: please translate</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -6171,7 +6363,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D211" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Blank: please supply,Draft: please check,Checked in the field,Needs discussion"</formula1>
+      <formula1>"English placeholder: please translate,Draft: please check,Checked in the field,Needs discussion"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6200,7 +6392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Column A is the English. Fill in or correct column B (Hindi) and column C (Punjabi). Yellow cells are blank because I was not sure of the local wording.</t>
+          <t>Column A is the English. Fill in or correct column B (Hindi) and column C (Punjabi). Yellow cells still show the English word because I was not sure of the local wording; please replace it.</t>
         </is>
       </c>
     </row>

</xml_diff>